<commit_message>
Manual data structure defintion added
</commit_message>
<xml_diff>
--- a/01_data_model/01_code_lists/01_general_codelists/input/code_lists_skeletons.xlsx
+++ b/01_data_model/01_code_lists/01_general_codelists/input/code_lists_skeletons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanniejo\Documents_local\01_dataplatform\021_SVbevraging\01_code\01_data_model\01_code_lists\01_general_codelists\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD98ED37-21BE-4EDC-9582-F2804FD618DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B86452-B65E-42F3-B7EA-3353D97ED26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="17172" windowWidth="23256" windowHeight="13176" firstSheet="28" activeTab="32" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="21" activeTab="32" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="agecat4" sheetId="1" r:id="rId1"/>
@@ -45,20 +45,21 @@
     <sheet name="roa" sheetId="32" r:id="rId30"/>
     <sheet name="satisf" sheetId="33" r:id="rId31"/>
     <sheet name="satsc" sheetId="34" r:id="rId32"/>
-    <sheet name="sex" sheetId="35" r:id="rId33"/>
-    <sheet name="strustfr" sheetId="36" r:id="rId34"/>
-    <sheet name="strusthp" sheetId="37" r:id="rId35"/>
-    <sheet name="strusttr" sheetId="38" r:id="rId36"/>
-    <sheet name="urbandgr" sheetId="39" r:id="rId37"/>
-    <sheet name="urbanlvl" sheetId="40" r:id="rId38"/>
-    <sheet name="yesno" sheetId="41" r:id="rId39"/>
+    <sheet name="semester" sheetId="44" r:id="rId33"/>
+    <sheet name="sex" sheetId="35" r:id="rId34"/>
+    <sheet name="strustfr" sheetId="36" r:id="rId35"/>
+    <sheet name="strusthp" sheetId="37" r:id="rId36"/>
+    <sheet name="strusttr" sheetId="38" r:id="rId37"/>
+    <sheet name="urbandgr" sheetId="39" r:id="rId38"/>
+    <sheet name="urbanlvl" sheetId="40" r:id="rId39"/>
+    <sheet name="yesno" sheetId="41" r:id="rId40"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="270">
   <si>
     <t>valuen</t>
   </si>
@@ -859,6 +860,15 @@
   </si>
   <si>
     <t>fwrespdisp</t>
+  </si>
+  <si>
+    <t>semester1</t>
+  </si>
+  <si>
+    <t>semester2</t>
+  </si>
+  <si>
+    <t>semester</t>
   </si>
 </sst>
 </file>
@@ -902,10 +912,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4046,6 +4059,54 @@
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A05C2A0-1D11-4378-B412-5EB70C8925CB}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4157,7 +4218,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4363,7 +4424,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4569,7 +4630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4775,7 +4836,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4862,7 +4923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4908,198 +4969,6 @@
         <v>255</v>
       </c>
       <c r="C4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="4" width="10.42578125" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>262</v>
-      </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>97</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>98</v>
-      </c>
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>99</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5225,6 +5094,198 @@
         <v>0</v>
       </c>
       <c r="D8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>262</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>98</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>99</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
clean data function finished
</commit_message>
<xml_diff>
--- a/01_data_model/01_code_lists/01_general_codelists/input/code_lists_skeletons.xlsx
+++ b/01_data_model/01_code_lists/01_general_codelists/input/code_lists_skeletons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanniejo\Documents_local\01_dataplatform\021_SVbevraging\01_code\01_data_model\01_code_lists\01_general_codelists\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B86452-B65E-42F3-B7EA-3353D97ED26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9D8BFD-D1EF-4B86-9E93-C733E1D21F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="21" activeTab="32" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3960" yWindow="17172" windowWidth="23256" windowHeight="13176" firstSheet="18" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="agecat4" sheetId="1" r:id="rId1"/>
@@ -34,32 +34,33 @@
     <sheet name="hind" sheetId="21" r:id="rId19"/>
     <sheet name="liveenv" sheetId="22" r:id="rId20"/>
     <sheet name="liveenvb" sheetId="23" r:id="rId21"/>
-    <sheet name="month" sheetId="24" r:id="rId22"/>
-    <sheet name="respdevice" sheetId="26" r:id="rId23"/>
-    <sheet name="respdisp" sheetId="27" r:id="rId24"/>
-    <sheet name="fwrespdisp" sheetId="42" r:id="rId25"/>
-    <sheet name="respmode" sheetId="28" r:id="rId26"/>
-    <sheet name="respons" sheetId="29" r:id="rId27"/>
-    <sheet name="respqrurl" sheetId="30" r:id="rId28"/>
-    <sheet name="resptime" sheetId="31" r:id="rId29"/>
-    <sheet name="roa" sheetId="32" r:id="rId30"/>
-    <sheet name="satisf" sheetId="33" r:id="rId31"/>
-    <sheet name="satsc" sheetId="34" r:id="rId32"/>
-    <sheet name="semester" sheetId="44" r:id="rId33"/>
-    <sheet name="sex" sheetId="35" r:id="rId34"/>
-    <sheet name="strustfr" sheetId="36" r:id="rId35"/>
-    <sheet name="strusthp" sheetId="37" r:id="rId36"/>
-    <sheet name="strusttr" sheetId="38" r:id="rId37"/>
-    <sheet name="urbandgr" sheetId="39" r:id="rId38"/>
-    <sheet name="urbanlvl" sheetId="40" r:id="rId39"/>
-    <sheet name="yesno" sheetId="41" r:id="rId40"/>
+    <sheet name="contact" sheetId="45" r:id="rId22"/>
+    <sheet name="month" sheetId="24" r:id="rId23"/>
+    <sheet name="respdevice" sheetId="26" r:id="rId24"/>
+    <sheet name="respdisp" sheetId="27" r:id="rId25"/>
+    <sheet name="fwrespdisp" sheetId="42" r:id="rId26"/>
+    <sheet name="respmode" sheetId="28" r:id="rId27"/>
+    <sheet name="respons" sheetId="29" r:id="rId28"/>
+    <sheet name="respqrurl" sheetId="30" r:id="rId29"/>
+    <sheet name="resptime" sheetId="31" r:id="rId30"/>
+    <sheet name="roa" sheetId="32" r:id="rId31"/>
+    <sheet name="satisf" sheetId="33" r:id="rId32"/>
+    <sheet name="satsc" sheetId="34" r:id="rId33"/>
+    <sheet name="semester" sheetId="44" r:id="rId34"/>
+    <sheet name="sex" sheetId="35" r:id="rId35"/>
+    <sheet name="strustfr" sheetId="36" r:id="rId36"/>
+    <sheet name="strusthp" sheetId="37" r:id="rId37"/>
+    <sheet name="strusttr" sheetId="38" r:id="rId38"/>
+    <sheet name="urbandgr" sheetId="39" r:id="rId39"/>
+    <sheet name="urbanlvl" sheetId="40" r:id="rId40"/>
+    <sheet name="yesno" sheetId="41" r:id="rId41"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="277">
   <si>
     <t>valuen</t>
   </si>
@@ -869,6 +870,27 @@
   </si>
   <si>
     <t>semester</t>
+  </si>
+  <si>
+    <t>answer</t>
+  </si>
+  <si>
+    <t>invitation</t>
+  </si>
+  <si>
+    <t>reminder_1</t>
+  </si>
+  <si>
+    <t>reminder_2</t>
+  </si>
+  <si>
+    <t>closing_paper</t>
+  </si>
+  <si>
+    <t>closing_online</t>
+  </si>
+  <si>
+    <t>contact</t>
   </si>
 </sst>
 </file>
@@ -2774,6 +2796,85 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5640D40A-4D2B-4B13-ACEF-D24F97300102}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>273</v>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2979,7 +3080,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3033,7 +3134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3164,7 +3265,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5AF9561-CE27-4632-8A57-56551249D738}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3184,8 +3285,8 @@
       <c r="A2">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B2" t="s">
-        <v>156</v>
+      <c r="B2" s="2" t="s">
+        <v>270</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -3273,7 +3374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3316,7 +3417,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3359,7 +3460,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3394,60 +3495,6 @@
         <v>174</v>
       </c>
       <c r="C3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>176</v>
-      </c>
-      <c r="C2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3582,6 +3629,60 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3689,7 +3790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3852,7 +3953,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4058,7 +4159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A05C2A0-1D11-4378-B412-5EB70C8925CB}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4106,7 +4207,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4218,7 +4319,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4424,7 +4525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4630,7 +4731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4836,7 +4937,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4915,60 +5016,6 @@
         <v>251</v>
       </c>
       <c r="C7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>253</v>
-      </c>
-      <c r="C2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>254</v>
-      </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>255</v>
-      </c>
-      <c r="C4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5103,6 +5150,60 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>